<commit_message>
updated several timeseries for NA, added filter option for timeseries
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file.xlsx
+++ b/Conversion Script/Set_filter_file.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Sector_selection" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Year_selection" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Rounding_thresholds" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Timeseries_selection" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="Fuels">#REF!</definedName>
@@ -2109,6 +2110,272 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Timeseries</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Timeseries selected</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TS_COOL_LOW</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TS_HEAT_HIGH</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TS_HEAT_LOW</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TS_HP_AIRSOURCE</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TS_HP_GROUNDSOURCE</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TS_HYDRO_ROR</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TS_LOAD</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TS_MOBILITY_PSNG</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TS_POWER_BEVS</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TS_POWER_BUILDINGS_COOLING</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TS_POWER_BUILDINGS_HEAT</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TS_POWER_DATACENTER</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TS_POWER_HYDROGEN</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TS_PV_AVG</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TS_PV_INF</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TS_PV_OPT</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TS_PV_ROOFTOP</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TS_PV_TRA</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TS_WIND_OFFSHORE</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TS_WIND_OFFSHORE_DEEP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TS_WIND_OFFSHORE_SHALLOW</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TS_WIND_ONSHORE_AVG</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TS_WIND_ONSHORE_INF</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TS_WIND_ONSHORE_OPT</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
added EGS with four price regions
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file.xlsx
+++ b/Conversion Script/Set_filter_file.xlsx
@@ -2382,7 +2382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B154"/>
+  <dimension ref="A1:B158"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3927,6 +3927,46 @@
         </is>
       </c>
       <c r="B154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>P_EGS_R1</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>P_EGS_R2</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>P_EGS_R3</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>P_EGS_R4</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>